<commit_message>
uploading sample student code and update pdf
</commit_message>
<xml_diff>
--- a/bond-assignment/data/BondPrices.xlsx
+++ b/bond-assignment/data/BondPrices.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tekampa/Library/CloudStorage/Dropbox/WO/TEACHING/Columbia/FinancialEconomics/AI_Project/FinEcon-instructor/bond-assignment/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61A0ADF-C1AA-2C4A-BF98-92ABCE5476B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF49FA34-953B-364E-B3D7-E987323ECF03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="760" windowWidth="28860" windowHeight="18100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="760" windowWidth="29560" windowHeight="19120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Price History" sheetId="2" r:id="rId1"/>
@@ -425,11 +425,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{858F3FAE-D928-462F-9C56-7F847EE233D1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD022E82-72C4-471E-B777-6231629E9CBA}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F243"/>
+  <dimension ref="A1:F255"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="8.5" customWidth="1"/>
@@ -5265,6 +5265,246 @@
         <v>102.26900000000001</v>
       </c>
     </row>
+    <row r="244" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A244" s="3">
+        <v>46248</v>
+      </c>
+      <c r="B244" s="4">
+        <v>99.769000000000005</v>
+      </c>
+      <c r="C244" s="4">
+        <v>98.471000000000004</v>
+      </c>
+      <c r="D244" s="4">
+        <v>96.313000000000002</v>
+      </c>
+      <c r="E244" s="4">
+        <v>86.772000000000006</v>
+      </c>
+      <c r="F244" s="4">
+        <v>101.995</v>
+      </c>
+    </row>
+    <row r="245" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A245" s="5">
+        <v>46251</v>
+      </c>
+      <c r="B245" s="6">
+        <v>99.504999999999995</v>
+      </c>
+      <c r="C245" s="6">
+        <v>98.480999999999995</v>
+      </c>
+      <c r="D245" s="6">
+        <v>96.088999999999999</v>
+      </c>
+      <c r="E245" s="6">
+        <v>86.614999999999995</v>
+      </c>
+      <c r="F245" s="6">
+        <v>101.813</v>
+      </c>
+    </row>
+    <row r="246" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A246" s="3">
+        <v>46252</v>
+      </c>
+      <c r="B246" s="4">
+        <v>99.474999999999994</v>
+      </c>
+      <c r="C246" s="4">
+        <v>98.411000000000001</v>
+      </c>
+      <c r="D246" s="4">
+        <v>96.003</v>
+      </c>
+      <c r="E246" s="4">
+        <v>86.626999999999995</v>
+      </c>
+      <c r="F246" s="4">
+        <v>101.738</v>
+      </c>
+    </row>
+    <row r="247" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A247" s="5">
+        <v>46253</v>
+      </c>
+      <c r="B247" s="6">
+        <v>99.953999999999994</v>
+      </c>
+      <c r="C247" s="6">
+        <v>98.436999999999998</v>
+      </c>
+      <c r="D247" s="6">
+        <v>96.491</v>
+      </c>
+      <c r="E247" s="6">
+        <v>86.71</v>
+      </c>
+      <c r="F247" s="6">
+        <v>102.18300000000001</v>
+      </c>
+    </row>
+    <row r="248" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A248" s="3">
+        <v>46254</v>
+      </c>
+      <c r="B248" s="4">
+        <v>99.54</v>
+      </c>
+      <c r="C248" s="4">
+        <v>98.135000000000005</v>
+      </c>
+      <c r="D248" s="4">
+        <v>96.072999999999993</v>
+      </c>
+      <c r="E248" s="4">
+        <v>86.533000000000001</v>
+      </c>
+      <c r="F248" s="4">
+        <v>101.80200000000001</v>
+      </c>
+    </row>
+    <row r="249" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A249" s="5">
+        <v>46255</v>
+      </c>
+      <c r="B249" s="6">
+        <v>99.441000000000003</v>
+      </c>
+      <c r="C249" s="6">
+        <v>98.31</v>
+      </c>
+      <c r="D249" s="6">
+        <v>96.180999999999997</v>
+      </c>
+      <c r="E249" s="6">
+        <v>86.475999999999999</v>
+      </c>
+      <c r="F249" s="6">
+        <v>101.185</v>
+      </c>
+    </row>
+    <row r="250" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A250" s="3">
+        <v>46258</v>
+      </c>
+      <c r="B250" s="4">
+        <v>99.578999999999994</v>
+      </c>
+      <c r="C250" s="4">
+        <v>98.475999999999999</v>
+      </c>
+      <c r="D250" s="4">
+        <v>96.257000000000005</v>
+      </c>
+      <c r="E250" s="4">
+        <v>86.494</v>
+      </c>
+      <c r="F250" s="4">
+        <v>101.34</v>
+      </c>
+    </row>
+    <row r="251" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A251" s="5">
+        <v>46259</v>
+      </c>
+      <c r="B251" s="6">
+        <v>100.04300000000001</v>
+      </c>
+      <c r="C251" s="6">
+        <v>98.480999999999995</v>
+      </c>
+      <c r="D251" s="6">
+        <v>96.754999999999995</v>
+      </c>
+      <c r="E251" s="6">
+        <v>86.8</v>
+      </c>
+      <c r="F251" s="6">
+        <v>102.142</v>
+      </c>
+    </row>
+    <row r="252" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A252" s="3">
+        <v>46260</v>
+      </c>
+      <c r="B252" s="4">
+        <v>99.924000000000007</v>
+      </c>
+      <c r="C252" s="4">
+        <v>98.488</v>
+      </c>
+      <c r="D252" s="4">
+        <v>96.634</v>
+      </c>
+      <c r="E252" s="4">
+        <v>86.680999999999997</v>
+      </c>
+      <c r="F252" s="4">
+        <v>102.074</v>
+      </c>
+    </row>
+    <row r="253" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A253" s="5">
+        <v>46261</v>
+      </c>
+      <c r="B253" s="6">
+        <v>99.813000000000002</v>
+      </c>
+      <c r="C253" s="6">
+        <v>98.55</v>
+      </c>
+      <c r="D253" s="6">
+        <v>96.575999999999993</v>
+      </c>
+      <c r="E253" s="6">
+        <v>86.715999999999994</v>
+      </c>
+      <c r="F253" s="6">
+        <v>102.04</v>
+      </c>
+    </row>
+    <row r="254" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A254" s="3">
+        <v>46262</v>
+      </c>
+      <c r="B254" s="4">
+        <v>99.41</v>
+      </c>
+      <c r="C254" s="4">
+        <v>98.442999999999998</v>
+      </c>
+      <c r="D254" s="4">
+        <v>96.221999999999994</v>
+      </c>
+      <c r="E254" s="4">
+        <v>86.509</v>
+      </c>
+      <c r="F254" s="4">
+        <v>101.727</v>
+      </c>
+    </row>
+    <row r="255" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A255" s="5">
+        <v>46265</v>
+      </c>
+      <c r="B255" s="6">
+        <v>99.346000000000004</v>
+      </c>
+      <c r="C255" s="6">
+        <v>98.460999999999999</v>
+      </c>
+      <c r="D255" s="6">
+        <v>95.988</v>
+      </c>
+      <c r="E255" s="6">
+        <v>86.46</v>
+      </c>
+      <c r="F255" s="6">
+        <v>101.64700000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>